<commit_message>
docs(secs): commit the workbook content 413df2f was supposed to carry
413df2f recorded only the git mv. The `git add` that should have staged the
edits listed both the old and the new path, the old one no longer existed, and
git aborted the whole command on that pathspec - so the commit went in as a
100% rename with the 20260805 bytes still inside. The content described in
413df2f's message is in this commit.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/SECS/SECS_GEM功能_HandlerV1_20260810.xlsx
+++ b/docs/SECS/SECS_GEM功能_HandlerV1_20260810.xlsx
@@ -1015,8 +1015,9 @@
  &lt;U4 [1] 1003&gt;
 &gt;
 .
-[20260805] 已實作。S1F3 -&gt; S1F4 回 L,n{SV 值}。⚠ 兩點請注意(與第 8 項 S2F13 / S2F14 同構)：(1) S1F4 的酬載依 SEMI E5 不回 SVID，請以「請求的順序」對位取值；本機未登錄的 SVID 回一個零長度項目(不是錯誤)，故 L 長度恆等於請求筆數、欄位不會位移。(2) 若送 &lt;L[0]&gt; 全查，回覆的 67 個值是本機的註冊順序，不是號碼遞增 —— 本檔「SVID」工作表為便於閱讀採號碼遞增排序，⚠ 請勿用該表的列序對位。實際註冊順序如下，前段 31 個：1001、1003、1021、1027、4、9、3、1002、1009、1006、1007、1008、1011、1101、1102、1103、1104、1105、1259、1260、1261、1517、37010、1518、1501、2758、2759、2760、2761、2762、2763；AMR 段 36 個：38219、38220、38221、38202、38222、38228、38203、38223、38229、38204、38224、38230、38205、38225、38231、38234、38206、38226、38232、38235、38207、38227、38233、38236、38199、38237、38240、38243、38200、38238、38241、38244、38201、38239、38242、38245(每個 Auto 站的 Bin Setting 緊跟在該站的 Carrier / Tray / Device 之後，不是另起一輪)，合計 67 筆。⚠ 建議貴端一律指名 SVID、不要送 &lt;L[0]&gt; —— 註冊順序會隨韌體改版而變動，指名取值才不受影響。⚠ 另請注意：單筆請求的指名清單上限為 512 筆，超過的部分會被靜默截斷(S1F3 / S1F11 / S1F23 / S2F13 四支相同)，此時回覆的 L 長度會小於請求筆數；本機只有 67 個 SVID，正常使用不會觸及此上限。
-〔20260805 韌體修正：共用解析器〕先前若請求清單中有一筆是**零長度的非 ASCII 型別**(例如 &lt;F8[0]&gt;)、或本機不支援的型別(U8 / I8 / BINARY)，該筆會卡在解析佇列最前端，導致其後的每一格都重複讀到同一筆壞資料、全部回零長度或 0。現已修正：該筆會被完整跳過，只有那一格回零長度，**其後各格的對位完全不受影響**。⚠ 這也是本表「不回號碼、請以請求順序對位取值」與「L 長度恆等於請求筆數、欄位不會位移」兩項承諾自本版起才**無條件**成立的原因 —— 在此之前，只要請求中夾了一顆本機讀不出的項目，該承諾就會失效。貴端一律以 ASCII 或本表宣告的型別送出號碼，即不會觸發此情形。</t>
+[20260805] 已實作。S1F3 -&gt; S1F4 回 L,n{SV 值}。⚠ 兩點請注意(與第 8 項 S2F13 / S2F14 同構)：(1) S1F4 的酬載依 SEMI E5 不回 SVID，請以「請求的順序」對位取值；本機未登錄的 SVID 回一個零長度項目(不是錯誤)，故 L 長度恆等於請求筆數、欄位不會位移。(2) 若送 &lt;L[0]&gt; 全查，回覆的 73 個值是本機的註冊順序，不是號碼遞增 —— 本檔「SVID」工作表為便於閱讀採號碼遞增排序，⚠ 請勿用該表的列序對位。實際註冊順序如下，前段 37 個：1001、1003、1021、1027、4、9、3、1002、1009、1006、1007、1008、1011、1101、1102、1103、1104、1105、1259、1260、1261、38237、38238、38239、38249、38250、38251、1517、37010、1518、1501、2758、2759、2760、2761、2762、2763；AMR 段 36 個：38219、38220、38221、38202、38222、38228、38203、38223、38229、38204、38224、38230、38205、38225、38231、38234、38206、38226、38232、38235、38207、38227、38233、38236、38199、38246、38240、38243、38200、38247、38241、38244、38201、38248、38242、38245(每個 Auto 站的 Bin Setting 緊跟在該站的 Carrier / Tray / Device 之後，不是另起一輪)，合計 73 筆。⚠ 建議貴端一律指名 SVID、不要送 &lt;L[0]&gt; —— 註冊順序會隨韌體改版而變動，指名取值才不受影響。⚠ 另請注意：單筆請求的指名清單上限為 512 筆，超過的部分會被靜默截斷(S1F3 / S1F11 / S1F23 / S2F13 四支相同)，此時回覆的 L 長度會小於請求筆數；本機只有 73 個 SVID，正常使用不會觸及此上限。
+〔20260805 韌體修正：共用解析器〕先前若請求清單中有一筆是**零長度的非 ASCII 型別**(例如 &lt;F8[0]&gt;)、或本機不支援的型別(U8 / I8 / BINARY)，該筆會卡在解析佇列最前端，導致其後的每一格都重複讀到同一筆壞資料、全部回零長度或 0。現已修正：該筆會被完整跳過，只有那一格回零長度，**其後各格的對位完全不受影響**。⚠ 這也是本表「不回號碼、請以請求順序對位取值」與「L 長度恆等於請求筆數、欄位不會位移」兩項承諾自本版起才**無條件**成立的原因 —— 在此之前，只要請求中夾了一顆本機讀不出的項目，該承諾就會失效。貴端一律以 ASCII 或本表宣告的型別送出號碼，即不會觸發此情形。
+〔20260810 追加項〕本版新增 6 個 SVID(38237-38239 Record Auto 1-3 Tray Count、38249-38251 Record Auto 4-6 Tray Count)，且 AMR AUTO4/5/6 Tray Count 由 38237-38239 改號為 38246-38248，故全查筆數由 67 增為 73，上列註冊順序已是本版順序。⚠ 語意改變的三個號碼請務必參閱「SVID」工作表表尾註 (e)。</t>
         </is>
       </c>
     </row>
@@ -1045,7 +1046,7 @@
   &lt;L [0] 
   &gt;
 .
-[20260805] 已實作。S1F11 -&gt; S1F12 回 L,n{L,3{U4 SVID, A SVNAME, A UNITS}}。⚠ 三點請注意：(1) 與 S1F4 / S2F14 不同，S1F12 每一筆都帶 SVID，貴端可直接以 SVID 對號取值，不需依請求順序對位；本機未登錄的 SVID 回 {SVID, '', ''}(名稱與單位皆為零長度，不是錯誤)。(2) 若送 &lt;L[0]&gt; 全查，回覆的 67 筆順序是本機的註冊順序，不是號碼遞增 —— 本檔「SVID」工作表採號碼遞增排序，⚠ 請勿用它推斷回覆順序；完整註冊順序見第 2 項 S1F3 的說明。(3) 指名清單與 &lt;L[0]&gt; 全查皆受「單筆請求最多 512 筆」的上限，超過的部分會被靜默截斷(S1F3 / S1F11 / S1F23 / S2F13 四支相同)；本機目前只有 67 個 SVID，故全查不會觸及此上限。
+[20260805] 已實作。S1F11 -&gt; S1F12 回 L,n{L,3{U4 SVID, A SVNAME, A UNITS}}。⚠ 三點請注意：(1) 與 S1F4 / S2F14 不同，S1F12 每一筆都帶 SVID，貴端可直接以 SVID 對號取值，不需依請求順序對位；本機未登錄的 SVID 回 {SVID, '', ''}(名稱與單位皆為零長度，不是錯誤)。(2) 若送 &lt;L[0]&gt; 全查，回覆的 73 筆順序是本機的註冊順序，不是號碼遞增 —— 本檔「SVID」工作表採號碼遞增排序，⚠ 請勿用它推斷回覆順序；完整註冊順序見第 2 項 S1F3 的說明。(3) 指名清單與 &lt;L[0]&gt; 全查皆受「單筆請求最多 512 筆」的上限，超過的部分會被靜默截斷(S1F3 / S1F11 / S1F23 / S2F13 四支相同)；本機目前只有 73 個 SVID，故全查不會觸及此上限。
 〔20260805 韌體修正：共用解析器〕先前若請求清單中有一筆是**零長度的非 ASCII 型別**(例如 &lt;F8[0]&gt;)、或本機不支援的型別(U8 / I8 / BINARY)，該筆會卡在解析佇列最前端，導致其後的每一格都重複讀到同一筆壞資料、全部回零長度或 0。現已修正：該筆會被完整跳過，只有那一格回零長度，**其後各格的對位完全不受影響**。⚠ 這也是本表「不回號碼、請以請求順序對位取值」與「L 長度恆等於請求筆數、欄位不會位移」兩項承諾自本版起才**無條件**成立的原因 —— 在此之前，只要請求中夾了一顆本機讀不出的項目，該承諾就會失效。貴端一律以 ASCII 或本表宣告的型別送出號碼，即不會觸發此情形。</t>
         </is>
       </c>
@@ -1287,12 +1288,12 @@
       <c r="E13" s="3" t="inlineStr">
         <is>
           <t>Define AMR related Report:'S2F33' W
-  &lt;L [2] 
+  &lt;L [2]
     &lt;U4 [1] 1&gt;
-    &lt;L [1] 
-      &lt;L [2] 
+    &lt;L [1]
+      &lt;L [2]
         &lt;U4 [1] 2000&gt;
-        &lt;L [7] 
+        &lt;L [7]
           &lt;U4 [1] 38202&gt; #Load port carrier ID
           &lt;U4 [1] 38205&gt; #Auto1 carrier ID
           &lt;U4 [1] 38206&gt; #Auto2 carrier ID
@@ -1305,7 +1306,14 @@
     &gt;
   &gt;
 .
-[20260805] 已實作。報表定義存於機台 system\EventReportDef.ini，開機時載入並疊加在本機內建報表之上，故貴端以 S2F33 定義的報表(RPTID 與其 SVID 清單)在復電後仍然存在。DRACK：0=受理 / 1=空間不足(單一封包最多 64 張報表、每張報表最多 192 個 SVID) / 2=封包格式錯誤 / 3=該 RPTID 是本機內建報表(RPTID 1-7)，不接受重新定義。本機不使用 DRACK=4。⚠ 刪除方式：整個報表清單送空(即 &lt;L[2]{DATAID, L[0]}&gt;)會刪除貴端先前以 S2F33 定義的全部報表並回 DRACK=0(本機內建的 1-7 不受影響)；單張報表的 SVID 清單送 L[0] 則只刪除該張報表。⚠ 容忍規則：本機不認識的 SVID 一律接受、不會回 DRACK=4(該號碼會寫進機台 SECS log 供比對)，但它在 S6F11 / S6F19 中會以零長度項目呈現 —— 報表的 L 長度不會縮短、其他欄位不會位移。⚠ 請先送 S2F33 定義報表，再送 S2F35 建立連結；順序顛倒時 S2F35 會靜默略過該連結(見第 12 項)。</t>
+[20260810 重大變更] 已實作。報表定義存於機台 system\EventReportDef.ini，開機時載入並疊加在本機內建報表之上，故貴端以 S2F33 定義的報表(RPTID 與其 SVID 清單)在復電後仍然存在。DRACK：0=受理 / 1=空間不足(單一封包最多 64 張報表、每張報表最多 192 個 SVID) / 2=封包格式錯誤 / 3=該 RPTID 是本機內建報表(RPTID 1-7)，不接受重新定義 / 4=封包內含本機未定義的 SVID。
+⚠⚠ 本版起改為嚴格驗證，取代 2026-07-27 起的容忍規則：封包內只要有一個本機未定義的 SVID，即回 DRACK=4 並整封拒絕 —— 一張報表都不會建立。拒絕是原子的：本機仍會把整封訊息解析到底(收訊路徑不失步)，在建立任何報表之前才回覆。此行為與 HT9045 一致。
+⚠ 舊行為(未定義的 SVID 一律接受、在 S6F11 以零長度項目呈現)自本版停用。改變原因：2026-08-07 現場實測顯示貴端定義的 7 張報表共引用 54 個本機未定義的 SVID，卻全部收到 DRACK=0，貴端因此無從得知那些資料永遠不會上傳。
+⚠ 對貴端的影響：請依本檔 SVID 頁的 73 個號碼重下 S2F33。已知貴端 RPTID 502 內含 SVID 1513 Tester On/Off —— 本機為 sorter、無測試機構、未註冊此號，故該張報表會整張被 DRACK=4 拒絕；其餘七個號碼本機都有，請將 1513 移除即可。
+⚠ 現場逃生口：system\General.ini [SECS] StrictReportValidation=0 可不重編韌體、暫時退回舊的容忍行為(預設值為 1)，供試機或量產不能等時使用。
+⚠ 刪除方式不變：整個報表清單送空(即 &lt;L[2]{DATAID, L[0]}&gt;)會刪除貴端先前以 S2F33 定義的全部報表並回 DRACK=0(本機內建的 1-7 不受影響)；單張報表的 SVID 清單送 L[0] 則只刪除該張報表。
+⚠ 請先送 S2F33 定義報表，再送 S2F35 建立連結；本版起順序顛倒會得到 LRACK=5(見第 12 項)。
+</t>
         </is>
       </c>
     </row>
@@ -1331,19 +1339,26 @@
       <c r="E14" s="3" t="inlineStr">
         <is>
           <t>AGVSupplement_Link_Report:'S2F35' W
-  &lt;L [2] 
+  &lt;L [2]
     &lt;U4 [1] 272&gt;
-    &lt;L [1] 
-      &lt;L [2] 
+    &lt;L [1]
+      &lt;L [2]
         &lt;U4 [1] 272&gt;
-        &lt;L [1] 
+        &lt;L [1]
           &lt;U4 [1] 2000&gt;
         &gt;
       &gt;
     &gt;
   &gt;
 .
-[20260805] 已實作。⚠ 事件→報表的連結為 session-only、不做持久化 —— 每次復電後全部連結退回本機出廠預設(292 個 CEID 中的 288 個連 Report 1，其餘四個 272 / 273 / 274 / 275 連本機內建的 AMR 專用報表)，貴端以 S2F35 建立的連結會消失。⚠ 請務必把「重新送出 S2F33 + S2F35(必要時再送 S2F37)」寫進貴端的復電 / 重連程序 —— S2F33 定義的報表本身有存檔，S2F35 的連結沒有，兩者不同，這是本機目前唯一的實質退化。LRACK：0=受理 / 2=封包格式錯誤，或超出容量(單一封包最多 64 個 CEID、每個 CEID 最多 32 個 RPTID)。本機不使用 LRACK=1 / 3 / 4 / 5。⚠ 三條容忍規則：(1) 連結到本機未註冊的 CEID 不會被拒絕 —— 該 CEID 會被建立並連結，但本機沒有對應的發射點，故永遠不會送出；(2) 連結到「當下尚未定義」的 RPTID 會被靜默略過，但整包仍回 LRACK=0 —— 故請勿以 LRACK=0 推斷連結一定成立，務必先送 S2F33 再送 S2F35，並可用 S1F23 / S1F24 回讀該 CEID 的 VID 清單確認；(3) 若某個 CEID 所送的 RPTID 全部都是未定義的，本機會保留該 CEID 原有的連結、不覆寫成空清單(避免整個事件的酬載被清空)；若貴端確實要解除連結，請把該 CEID 的 RPTID 清單明確送成 L[0]。⚠ 另：整個 CEID 清單送空(即 &lt;L[2]{DATAID, L[0]}&gt;)為 no-op，回 LRACK=0 但不會解除任何連結。</t>
+[20260810 重大變更] 已實作。⚠ 事件→報表的連結為 session-only、不做持久化 —— 每次復電後全部連結退回本機出廠預設(292 個 CEID 中的 288 個連 Report 1，其餘四個 272 / 273 / 274 / 275 連本機內建的 AMR 專用報表)，貴端以 S2F35 建立的連結會消失。⚠ 請務必把「重新送出 S2F33 + S2F35(必要時再送 S2F37)」寫進貴端的復電 / 重連程序 —— S2F33 定義的報表本身有存檔，S2F35 的連結沒有，兩者不同，這是本機目前唯一的實質退化。
+LRACK：0=受理 / 2=封包格式錯誤，或超出容量(單一封包最多 64 個 CEID、每個 CEID 最多 32 個 RPTID) / 4=封包內含本機未註冊的 CEID / 5=封包內含本機尚未定義的 RPTID。本機不使用 LRACK=1 / 3。
+⚠⚠ 本版起改為嚴格驗證，取代 2026-07-27 起的三條容忍規則：封包內只要有一個本機未註冊的 CEID 即回 LRACK=4；只要有一個尚未定義的 RPTID 即回 LRACK=5；兩者都是整封拒絕 —— 一條連結都不會建立。同一封包兩種錯誤都有時，先回報 CEID 錯誤(LRACK=4)，因為 CEID 是外層物件。拒絕同樣是原子且延後的：整封解析到底、在建立任何連結之前才回覆。此行為與 HT9045 一致。
+⚠ 舊行為自本版停用：(1) 連結到未註冊的 CEID 不再被建立，(2) 連結到未定義的 RPTID 不再被靜默略過。因此 LRACK=0 現在確實代表整包連結全部成立 —— 這是本次變更帶給貴端的主要好處。
+⚠ 順序要求因此成為硬性規定：務必先送 S2F33 定義報表、再送 S2F35，順序顛倒會得到 LRACK=5。仍可用 S1F23 / S1F24 回讀該 CEID 的 VID 清單做確認。
+⚠ 不變的兩點：整個 CEID 清單送空(即 &lt;L[2]{DATAID, L[0]}&gt;)仍為 no-op，回 LRACK=0 但不會解除任何連結；若貴端確實要解除某個 CEID 的連結，請把該 CEID 的 RPTID 清單明確送成 L[0]。
+⚠ 現場逃生口同 S2F33：system\General.ini [SECS] StrictReportValidation=0(預設 1)。
+</t>
         </is>
       </c>
     </row>
@@ -2559,7 +2574,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F72"/>
+  <dimension ref="A1:F79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5"/>
   <cols>
     <col width="6.5" bestFit="1" customWidth="1" style="22" min="1" max="1"/>
@@ -4376,7 +4391,7 @@
       </c>
       <c r="B60" s="40" t="inlineStr">
         <is>
-          <t>AMR AUTO4 Tray Count</t>
+          <t>Record Auto 1 Tray Count</t>
         </is>
       </c>
       <c r="C60" s="40" t="inlineStr">
@@ -4396,7 +4411,7 @@
       </c>
       <c r="F60" s="40" t="inlineStr">
         <is>
-          <t>取自 AUTO4 出料車的即時盤數。CEID 274 發出前先做最後一次快照，事件送出後歸零(車已被取走)。僅在 UseAMR=1 時維護，詳見表尾註 (a)。</t>
+          <t>AUTO1 本工單累計已產出的整盤數，於整盤自 AUTO1 出料完成時 +1(與該軌道 Unloadtray 事件 CEID 136 同一時點)。與 HT9045 SVID 38237 同號同義(HT9046LS V3.32.810_B01)。⚠ 清除時機：本機於 Lot Start 清零，非 HT9045 的 Lot End —— 因本機可同時掛最多 64 批，任一批 Lot End 都無法指認軌道計數器中的盤屬於哪一批；此點待貴端確認。⚠ 與 SVID 1103 Auto1 Count 不同：1103 數的是「當前盤内的 IC 顆數」，本號數的是「已完成的盤數」。〔20260810 新增：本號原為 AMR AUTO4 Tray Count，已讓位至 38246。〕</t>
         </is>
       </c>
     </row>
@@ -4406,7 +4421,7 @@
       </c>
       <c r="B61" s="40" t="inlineStr">
         <is>
-          <t>AMR AUTO5 Tray Count</t>
+          <t>Record Auto 2 Tray Count</t>
         </is>
       </c>
       <c r="C61" s="40" t="inlineStr">
@@ -4426,7 +4441,7 @@
       </c>
       <c r="F61" s="40" t="inlineStr">
         <is>
-          <t>取自 AUTO5 出料車的即時盤數。CEID 274 發出前先做最後一次快照，事件送出後歸零(車已被取走)。僅在 UseAMR=1 時維護，詳見表尾註 (a)。</t>
+          <t>AUTO2 本工單累計已產出的整盤數，於整盤自 AUTO2 出料完成時 +1(與該軌道 Unloadtray 事件 CEID 137 同一時點)。與 HT9045 SVID 38238 同號同義(HT9046LS V3.32.810_B01)。⚠ 清除時機：本機於 Lot Start 清零，非 HT9045 的 Lot End —— 因本機可同時掛最多 64 批，任一批 Lot End 都無法指認軌道計數器中的盤屬於哪一批；此點待貴端確認。⚠ 與 SVID 1104 Auto2 Count 不同：1104 數的是「當前盤内的 IC 顆數」，本號數的是「已完成的盤數」。〔20260810 新增：本號原為 AMR AUTO5 Tray Count，已讓位至 38247。〕</t>
         </is>
       </c>
     </row>
@@ -4436,7 +4451,7 @@
       </c>
       <c r="B62" s="40" t="inlineStr">
         <is>
-          <t>AMR AUTO6 Tray Count</t>
+          <t>Record Auto 3 Tray Count</t>
         </is>
       </c>
       <c r="C62" s="40" t="inlineStr">
@@ -4456,7 +4471,7 @@
       </c>
       <c r="F62" s="40" t="inlineStr">
         <is>
-          <t>取自 AUTO6 出料車的即時盤數。CEID 274 發出前先做最後一次快照，事件送出後歸零(車已被取走)。僅在 UseAMR=1 時維護，詳見表尾註 (a)。</t>
+          <t>AUTO3 本工單累計已產出的整盤數，於整盤自 AUTO3 出料完成時 +1(與該軌道 Unloadtray 事件 CEID 138 同一時點)。與 HT9045 SVID 38239 同號同義(HT9046LS V3.32.810_B01)。⚠ 清除時機：本機於 Lot Start 清零，非 HT9045 的 Lot End —— 因本機可同時掛最多 64 批，任一批 Lot End 都無法指認軌道計數器中的盤屬於哪一批；此點待貴端確認。⚠ 與 SVID 1105 Auto3 Count 不同：1105 數的是「當前盤内的 IC 顆數」，本號數的是「已完成的盤數」。〔20260810 新增：本號原為 AMR AUTO6 Tray Count，已讓位至 38248。〕</t>
         </is>
       </c>
     </row>
@@ -4641,30 +4656,217 @@
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="43" t="inlineStr">
-        <is>
-          <t>〔20260805 追加項：表尾註 (a)〕AMR 系列 SVID 38199-38245(共 36 個號碼)僅在 system\General.ini [HardwareInstall] UseAMR=1 時維護。UseAMR=0(本機出廠預設，也是一般量產模式)時這些值不再刷新，停留在開機初值(數值為 0、字串為零長度)；S1F3 仍可讀到，但內容沒有意義，請勿據以判斷機台實況。⚠ 一個例外：SVID 38202 Loader Carrier ID(身分盤 2D)的更新路徑不受 UseAMR 影響，因此 UseAMR=0 下只要走到身分盤讀碼流程，38202 仍會被更新並送出 CEID 275。其餘 35 個號碼確實只在 UseAMR=1 時維護。〔20260805 更正：本句原本指的是 38204；身分盤 2D 已改發布在 38202。〕</t>
+      <c r="A69" s="43" t="n">
+        <v>38246</v>
+      </c>
+      <c r="B69" s="40" t="inlineStr">
+        <is>
+          <t>AMR AUTO4 Tray Count</t>
+        </is>
+      </c>
+      <c r="C69" s="40" t="inlineStr">
+        <is>
+          <t>I4</t>
+        </is>
+      </c>
+      <c r="D69" s="40" t="inlineStr">
+        <is>
+          <t>trays</t>
+        </is>
+      </c>
+      <c r="E69" s="40" t="inlineStr">
+        <is>
+          <t>0 以上整數</t>
+        </is>
+      </c>
+      <c r="F69" s="40" t="inlineStr">
+        <is>
+          <t>取自 AUTO4 出料車的即時盤數。CEID 274 發出前先做最後一次快照，事件送出後歸零(車已被取走)。僅在 UseAMR=1 時維護，詳見表尾註 (a)。〔20260810 改號：本號原為 38237，因 HT9045 已將 38237 定義為 Record Auto 1 Tray Count，本機讓位改用 38246。舊號 38237 請改綁本號。〕</t>
         </is>
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="43" t="inlineStr">
+      <c r="A70" s="43" t="n">
+        <v>38247</v>
+      </c>
+      <c r="B70" s="40" t="inlineStr">
+        <is>
+          <t>AMR AUTO5 Tray Count</t>
+        </is>
+      </c>
+      <c r="C70" s="40" t="inlineStr">
+        <is>
+          <t>I4</t>
+        </is>
+      </c>
+      <c r="D70" s="40" t="inlineStr">
+        <is>
+          <t>trays</t>
+        </is>
+      </c>
+      <c r="E70" s="40" t="inlineStr">
+        <is>
+          <t>0 以上整數</t>
+        </is>
+      </c>
+      <c r="F70" s="40" t="inlineStr">
+        <is>
+          <t>取自 AUTO5 出料車的即時盤數。CEID 274 發出前先做最後一次快照，事件送出後歸零(車已被取走)。僅在 UseAMR=1 時維護，詳見表尾註 (a)。〔20260810 改號：本號原為 38238，因 HT9045 已將 38238 定義為 Record Auto 2 Tray Count，本機讓位改用 38247。舊號 38238 請改綁本號。〕</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="43" t="n">
+        <v>38248</v>
+      </c>
+      <c r="B71" s="40" t="inlineStr">
+        <is>
+          <t>AMR AUTO6 Tray Count</t>
+        </is>
+      </c>
+      <c r="C71" s="40" t="inlineStr">
+        <is>
+          <t>I4</t>
+        </is>
+      </c>
+      <c r="D71" s="40" t="inlineStr">
+        <is>
+          <t>trays</t>
+        </is>
+      </c>
+      <c r="E71" s="40" t="inlineStr">
+        <is>
+          <t>0 以上整數</t>
+        </is>
+      </c>
+      <c r="F71" s="40" t="inlineStr">
+        <is>
+          <t>取自 AUTO6 出料車的即時盤數。CEID 274 發出前先做最後一次快照，事件送出後歸零(車已被取走)。僅在 UseAMR=1 時維護，詳見表尾註 (a)。〔20260810 改號：本號原為 38239，因 HT9045 已將 38239 定義為 Record Auto 3 Tray Count，本機讓位改用 38248。舊號 38239 請改綁本號。〕</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="43" t="n">
+        <v>38249</v>
+      </c>
+      <c r="B72" s="40" t="inlineStr">
+        <is>
+          <t>Record Auto 4 Tray Count</t>
+        </is>
+      </c>
+      <c r="C72" s="40" t="inlineStr">
+        <is>
+          <t>I4</t>
+        </is>
+      </c>
+      <c r="D72" s="40" t="inlineStr">
+        <is>
+          <t>trays</t>
+        </is>
+      </c>
+      <c r="E72" s="40" t="inlineStr">
+        <is>
+          <t>0 以上整數</t>
+        </is>
+      </c>
+      <c r="F72" s="40" t="inlineStr">
+        <is>
+          <t>AUTO4 本工單累計已產出的整盤數，於整盤自 AUTO4 出料完成時 +1(與該軌道 Unloadtray 事件 CEID 145 同一時點)。⚠ HT9045 家族只組到 Auto1-3(38237-38239)，Auto4-6 無家族號可用，故 38249-38251 為本機擴充號。⚠ 清除時機：本機於 Lot Start 清零，非 HT9045 的 Lot End —— 因本機可同時掛最多 64 批，任一批 Lot End 都無法指認軌道計數器中的盤屬於哪一批；此點待貴端確認。⚠ 與 SVID 1259 Auto4 Count 不同：1259 數的是「當前盤内的 IC 顆數」，本號數的是「已完成的盤數」。</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="43" t="n">
+        <v>38250</v>
+      </c>
+      <c r="B73" s="40" t="inlineStr">
+        <is>
+          <t>Record Auto 5 Tray Count</t>
+        </is>
+      </c>
+      <c r="C73" s="40" t="inlineStr">
+        <is>
+          <t>I4</t>
+        </is>
+      </c>
+      <c r="D73" s="40" t="inlineStr">
+        <is>
+          <t>trays</t>
+        </is>
+      </c>
+      <c r="E73" s="40" t="inlineStr">
+        <is>
+          <t>0 以上整數</t>
+        </is>
+      </c>
+      <c r="F73" s="40" t="inlineStr">
+        <is>
+          <t>AUTO5 本工單累計已產出的整盤數，於整盤自 AUTO5 出料完成時 +1(與該軌道 Unloadtray 事件 CEID 146 同一時點)。⚠ HT9045 家族只組到 Auto1-3(38237-38239)，Auto4-6 無家族號可用，故 38249-38251 為本機擴充號。⚠ 清除時機：本機於 Lot Start 清零，非 HT9045 的 Lot End —— 因本機可同時掛最多 64 批，任一批 Lot End 都無法指認軌道計數器中的盤屬於哪一批；此點待貴端確認。⚠ 與 SVID 1260 Auto5 Count 不同：1260 數的是「當前盤内的 IC 顆數」，本號數的是「已完成的盤數」。</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="43" t="n">
+        <v>38251</v>
+      </c>
+      <c r="B74" s="40" t="inlineStr">
+        <is>
+          <t>Record Auto 6 Tray Count</t>
+        </is>
+      </c>
+      <c r="C74" s="40" t="inlineStr">
+        <is>
+          <t>I4</t>
+        </is>
+      </c>
+      <c r="D74" s="40" t="inlineStr">
+        <is>
+          <t>trays</t>
+        </is>
+      </c>
+      <c r="E74" s="40" t="inlineStr">
+        <is>
+          <t>0 以上整數</t>
+        </is>
+      </c>
+      <c r="F74" s="40" t="inlineStr">
+        <is>
+          <t>AUTO6 本工單累計已產出的整盤數，於整盤自 AUTO6 出料完成時 +1(與該軌道 Unloadtray 事件 CEID 147 同一時點)。⚠ HT9045 家族只組到 Auto1-3(38237-38239)，Auto4-6 無家族號可用，故 38249-38251 為本機擴充號。⚠ 清除時機：本機於 Lot Start 清零，非 HT9045 的 Lot End —— 因本機可同時掛最多 64 批，任一批 Lot End 都無法指認軌道計數器中的盤屬於哪一批；此點待貴端確認。⚠ 與 SVID 1261 Auto6 Count 不同：1261 數的是「當前盤内的 IC 顆數」，本號數的是「已完成的盤數」。</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="43" t="inlineStr">
+        <is>
+          <t>〔20260805 追加項：表尾註 (a)〕AMR 系列 SVID 38199-38251 之間(不連續，共 36 個號碼，不含 Record Auto 的 38237-38239 與 38249-38251)僅在 system\General.ini [HardwareInstall] UseAMR=1 時維護。UseAMR=0(本機出廠預設，也是一般量產模式)時這些值不再刷新，停留在開機初值(數值為 0、字串為零長度)；S1F3 仍可讀到，但內容沒有意義，請勿據以判斷機台實況。⚠ 一個例外：SVID 38202 Loader Carrier ID(身分盤 2D)的更新路徑不受 UseAMR 影響，因此 UseAMR=0 下只要走到身分盤讀碼流程，38202 仍會被更新並送出 CEID 275。其餘 35 個號碼確實只在 UseAMR=1 時維護。〔20260805 更正：本句原本指的是 38204；身分盤 2D 已改發布在 38202。〕</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="43" t="inlineStr">
         <is>
           <t>〔20260805 追加項：表尾註 (b)〕⚠ 身分盤 2D 的公布號碼為 SVID 38202 Loader Carrier ID，與 HT9045 一致 —— 貴端自訂報表 RPTID 2000 的第一格不需修改。本版之前該值放在 SVID 38204 Color Carrier ID(因為 Color 站才是實際讀 2D 的讀碼器)，依貴端 2026-08-05 的裁示「與 9045 對齊優先」已改回 38202;CEID 275 內建的 Report 7 亦隨之改為僅含 38202。⚠ 連帶影響：SVID 38204 自此不再有任何寫入者、恆回零長度，請勿再引用。</t>
         </is>
       </c>
     </row>
-    <row r="71">
-      <c r="A71" s="43" t="inlineStr">
+    <row r="77">
+      <c r="A77" s="43" t="inlineStr">
         <is>
           <t>〔20260805 追加項：表尾註 (c)〕⚠ 下列六個號碼只是為了對齊站別向量而註冊，本機不維護其值，恆為 0 或零長度字串：38203(Empty Carrier ID)、38204(Color Carrier ID，自 20260805 起，見表尾註 (b))、38223/38224(Empty/Color Tray Count)、38229/38230(Empty/Color Device Count)。原因是 Empty 與 Color 兩站完全由 sensor 與 TrayArm 驅動、不經 SECS，機構上也沒有疊盤計數器。CEID 272/274 的 Report 6 內這幾格同樣恆 0，請勿用來判斷實際盤數。</t>
         </is>
       </c>
     </row>
-    <row r="72">
-      <c r="A72" s="43" t="inlineStr">
+    <row r="78">
+      <c r="A78" s="43" t="inlineStr">
         <is>
           <t>[20260805] 表尾註 (d)：本表「型別」與「單位」兩欄即本機註冊時宣告的型別與單位，也就是 S1F11→S1F12 回覆中該 SVID 的單位欄內容；無單位者 S1F12 回零長度字串，本表以「—」表示。型別對照：ASCII=&lt;A&gt;、U1=&lt;U1&gt;、I4=&lt;I4&gt;、F8=&lt;F8&gt;。</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="43" t="inlineStr">
+        <is>
+          <t>〔20260810 追加項：表尾註 (e)〕⚠⚠ 本版有三個號碼的【語意改變】，不是只停用：38237 / 38238 / 38239 本版之前是 AMR AUTO4/5/6 Tray Count(出料車上的即時盤數)，本版起改為 HT9045 家族定義的 Record Auto 1/2/3 Tray Count(本工單累計出盤數)。兩者型別相同(I4)、數值都看起來合理，線上無法分辨，故在此明確告知。若貴端 host 在 2026-08-10 之前已將 38237-38239 綁為 AMR 車上盤數，請改綁 38246-38248。原因：HT9046LS V3.32.810_B01 於 2026-07-10 新增了 38237-38239 = Record Auto 1/2/3 Tray Count，家族號優先，本機原本占用該三號的 AMR 盤數讓位。</t>
         </is>
       </c>
     </row>

</xml_diff>